<commit_message>
1 Test case Added
</commit_message>
<xml_diff>
--- a/testdata/Cogmento-CRM_Web.xlsx
+++ b/testdata/Cogmento-CRM_Web.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" activeTab="1"/>
+    <workbookView windowWidth="19200" windowHeight="8000"/>
   </bookViews>
   <sheets>
     <sheet name="createNewContact" sheetId="1" r:id="rId1"/>
-    <sheet name="validateCreatedContact" sheetId="3" r:id="rId2"/>
+    <sheet name="createNewEvent" sheetId="3" r:id="rId2"/>
+    <sheet name="createNewDeal" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t>firstName</t>
   </si>
@@ -153,36 +154,103 @@
     <t>D:\\Automation_Redefined\\Cogmento-CRM-Web\\testdata\\img1.jpg</t>
   </si>
   <si>
-    <t>search</t>
-  </si>
-  <si>
-    <t>operator</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Equals</t>
+    <t>Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start Date
+</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>All Day</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>@@Str(10)</t>
+  </si>
+  <si>
+    <t>Meeting</t>
+  </si>
+  <si>
+    <t>@@Str(20)</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>closedate</t>
+  </si>
+  <si>
+    <t>probability</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>filterSearch</t>
+  </si>
+  <si>
+    <t>@@Str(8)</t>
+  </si>
+  <si>
+    <t>@@Str(4)</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>online</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="dd/mmm/yy"/>
+    <numFmt numFmtId="180" formatCode="[$-409]dddd\,mmmm\ d\,yyyy;@"/>
+    <numFmt numFmtId="181" formatCode="dd/mmm/yy"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.75"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -352,7 +420,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.25"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -682,144 +750,147 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -880,6 +951,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
+<customStorage xmlns="https://web.wps.cn/et/2018/main">
+  <book/>
+  <sheets/>
+</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1159,94 +1237,94 @@
     <col min="36" max="36" width="11.7272727272727" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:35">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="5" customFormat="1" spans="1:35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6"/>
-      <c r="AB1" s="6"/>
-      <c r="AC1" s="6"/>
-      <c r="AD1" s="6"/>
-      <c r="AE1" s="6"/>
-      <c r="AF1" s="6"/>
-      <c r="AG1" s="6"/>
-      <c r="AH1" s="6"/>
-      <c r="AI1" s="6"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="2" t="s">
@@ -1274,7 +1352,7 @@
       <c r="I2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="7" t="s">
         <v>34</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -1310,7 +1388,7 @@
       </c>
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
-      <c r="X2" s="5">
+      <c r="X2" s="8">
         <v>35756</v>
       </c>
       <c r="Y2" s="2" t="s">
@@ -1319,15 +1397,15 @@
       <c r="Z2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AA2" s="7"/>
-      <c r="AB2" s="7"/>
-      <c r="AC2" s="7"/>
-      <c r="AD2" s="7"/>
-      <c r="AE2" s="7"/>
-      <c r="AF2" s="7"/>
-      <c r="AG2" s="7"/>
-      <c r="AH2" s="7"/>
-      <c r="AI2" s="7"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10"/>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1341,32 +1419,147 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="11.8181818181818" customWidth="1"/>
+    <col min="2" max="2" width="22.0909090909091" customWidth="1"/>
+    <col min="3" max="3" width="22.8181818181818" customWidth="1"/>
+    <col min="5" max="5" width="11.5454545454545" customWidth="1"/>
+    <col min="6" max="6" width="10.8181818181818" customWidth="1"/>
+    <col min="7" max="7" width="7.45454545454545" customWidth="1"/>
+    <col min="8" max="8" width="15.1818181818182" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:8">
+      <c r="A1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="3">
+        <v>45879.1875</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45876.2291666667</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" display="xyz@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1"/>
+  <cols>
+    <col min="3" max="3" width="21.3636363636364" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="10.6363636363636" customWidth="1"/>
+    <col min="9" max="9" width="11.2727272727273" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>0</v>
+        <v>53</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>36</v>
+    <row r="2" spans="1:9">
+      <c r="A2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45836.625</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="2">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1000</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>